<commit_message>
vault backup: 2026-08-10 17:37:01
</commit_message>
<xml_diff>
--- a/工作交付文档/需求开发记录/assets/随州中心医院-住院病案附页-字段生成/V3366病案首页生成字段.xlsx
+++ b/工作交付文档/需求开发记录/assets/随州中心医院-住院病案附页-字段生成/V3366病案首页生成字段.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\76304\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\gitee\obsidian_qyc_book\工作交付文档\需求开发记录\assets\随州中心医院-住院病案附页-字段生成\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="29872" windowHeight="13335"/>
+    <workbookView windowWidth="27705" windowHeight="12975" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="随州中心医院病案首页新加字段" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="117">
   <si>
     <t>序号</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>查看依据</t>
+  </si>
+  <si>
+    <t>负责人</t>
   </si>
   <si>
     <t>是否急性ST段抬高型心肌梗死</t>
@@ -90,6 +93,13 @@
 （3）未执行：未在发病 12 小时内实施 PCI 或静脉溶栓。</t>
   </si>
   <si>
+    <t>入院记录，手术记录，操作记录，查房记录、日常病程记录
+召召了解一下？填写的入口条件</t>
+  </si>
+  <si>
+    <t>秦宇晨</t>
+  </si>
+  <si>
     <t>是否急性脑梗死</t>
   </si>
   <si>
@@ -124,11 +134,18 @@
 第 6、7、8、9 项自动填写“-”。</t>
   </si>
   <si>
+    <t>“肿瘤治疗前是否进行临床 TNM 分期“ 的区别</t>
+  </si>
+  <si>
     <t>肿瘤临床分期时间</t>
   </si>
   <si>
     <t>首先通过主诉和现病史判断患者此次住院是1、首次入院治疗肿瘤。2、非手术治疗后入院治疗、3、手术治疗后入院治疗。
 然后还要判断此次入院记录中的初步诊断或出院诊断中出院诊断总肿瘤TNM分期是在手术前还是手术后。</t>
+  </si>
+  <si>
+    <t>主诉和现病史（入院记录）
+召召了解一下？填写的入口条件？ VS “肿瘤治疗前是否进行临床 TNM 分期“ 的区别</t>
   </si>
   <si>
     <t>临床TNM分期-T</t>
@@ -145,6 +162,12 @@
 不确定有无远处转移。</t>
   </si>
   <si>
+    <t>入院记录、查房记录、出院记录  /抽取任务，不要模型去判断</t>
+  </si>
+  <si>
+    <t>帮主</t>
+  </si>
+  <si>
     <t>临床TNM分期-N</t>
   </si>
   <si>
@@ -154,7 +177,18 @@
     <t>肝癌临床CNLC分期</t>
   </si>
   <si>
+    <t>入院记录、查房记录、出院记录
+召召了解一下？填写的入口条件？确定具体的肿瘤类型范围，取值范围(/抽取任务)</t>
+  </si>
+  <si>
+    <t>杨总</t>
+  </si>
+  <si>
     <t>宫颈癌临床分期（FIGO 2018版）</t>
+  </si>
+  <si>
+    <t>入院记录、查房记录、出院记录
+召召了解一下？填写的入口条件？确定具体的肿瘤类型范围, 取值范围(/抽取任务)</t>
   </si>
   <si>
     <t>子宫内膜癌手术病理分期（FIGO 2009版）</t>
@@ -170,13 +204,23 @@
 否则该项填“2”，第“11、12、13”项填报为“-”。</t>
   </si>
   <si>
+    <t>召召了解一下？</t>
+  </si>
+  <si>
     <t>住院期间是否进行VTE评估</t>
   </si>
   <si>
     <t>直接从病历识别评估结果，入院记录（辅助检查）</t>
   </si>
   <si>
+    <t xml:space="preserve">入院记录 </t>
+  </si>
+  <si>
     <t>风险评估等级-手术患者</t>
+  </si>
+  <si>
+    <t>入院记录
+召召了解一下？如何判断使用了那个评估量表，取值范围不一样</t>
   </si>
   <si>
     <t>风险评估等级-非手术患者</t>
@@ -196,6 +240,9 @@
 （4）无：未做相应预防措施。</t>
   </si>
   <si>
+    <t>查房记录</t>
+  </si>
+  <si>
     <t>是否使用抗菌药物</t>
   </si>
   <si>
@@ -208,12 +255,19 @@
     <t>参考病历质控系统中制作的抗菌药物目录，是否病原学送检的提示词</t>
   </si>
   <si>
+    <t>病案质控中，我们做过了，有抗菌药物的收费项触发，查看医疗文本里是否有送检的相关描述</t>
+  </si>
+  <si>
     <t>有无输血反应</t>
   </si>
   <si>
     <t>参考病历质控系统有有无输血的判断。不良反应从病程记录+查房记录判断</t>
   </si>
   <si>
+    <t>日常病程记录，查房记录
+召召了解一下？ 入口判断是否输过血（收费项目判断：红细胞、血小板、血浆、全血、自体回收、其他）</t>
+  </si>
+  <si>
     <t>红细胞</t>
   </si>
   <si>
@@ -295,6 +349,9 @@
     <t>使用护理记录生成。若该项目填“1”，下一项必填；若该项目填“2”，下一项填“-”；</t>
   </si>
   <si>
+    <t>护理记录</t>
+  </si>
+  <si>
     <t>跌倒/坠床原因</t>
   </si>
   <si>
@@ -314,6 +371,9 @@
   </si>
   <si>
     <t>首页年龄小于28天时，根据入院记录生成</t>
+  </si>
+  <si>
+    <t>入院记录 （1.正常新生儿 2.早产儿 3.有疾病新生儿 4.非无菌分娩 5.其它）</t>
   </si>
   <si>
     <t>治疗转归</t>
@@ -336,16 +396,25 @@
     <t>有疑难病例讨论记录</t>
   </si>
   <si>
+    <t>原先病案文本类型分类已做过</t>
+  </si>
+  <si>
     <t>是否是MDT病例</t>
   </si>
   <si>
     <t>有多学科讨论记录</t>
   </si>
   <si>
+    <t>（疑难病例讨论记录-&gt;多学科讨论记录），博士建议直接关键词区分</t>
+  </si>
+  <si>
     <t>是否是日间手术病例</t>
   </si>
   <si>
     <t>有日间病房入、出院记录或日间手术记录、日间病房入住知情同意书</t>
+  </si>
+  <si>
+    <t>召召了解一下，看一下医院的标题名称就能做，查一下《24小时出入院记录》是否就是日间手术病例，限制条件：1.住院是否小于等于1天的； 2.有手术或者操作（化疗？） 3. 大模型判断一下是否做了手术</t>
   </si>
   <si>
     <t>诊断符合情况-出院与门诊</t>
@@ -556,7 +625,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -573,6 +642,12 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor theme="4" tint="0.799981688894314"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.8"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -1005,7 +1080,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1029,16 +1104,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1047,89 +1122,89 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1166,6 +1241,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1178,62 +1256,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1241,8 +1313,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1768,18 +1840,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:E45"/>
-  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:F45"/>
+  <sheetFormatPr defaultColWidth="9.025" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="9.02654867256637" style="19"/>
-    <col min="2" max="2" width="20.0884955752212" style="19" customWidth="1"/>
-    <col min="3" max="3" width="10.2477876106195" style="19" customWidth="1"/>
-    <col min="4" max="4" width="96.9115044247788" customWidth="1"/>
-    <col min="5" max="5" width="28.787610619469" customWidth="1"/>
+    <col min="1" max="1" width="7.41666666666667" style="18" customWidth="1"/>
+    <col min="2" max="2" width="33.7916666666667" style="18" customWidth="1"/>
+    <col min="3" max="3" width="9.225" style="18" customWidth="1"/>
+    <col min="4" max="4" width="45.0916666666667" style="12" customWidth="1"/>
+    <col min="5" max="5" width="41.6333333333333" customWidth="1"/>
+    <col min="6" max="6" width="9.025" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" customFormat="1" spans="1:6">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -1789,622 +1862,750 @@
       <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="22" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" ht="40.5" spans="1:5">
-      <c r="A2" s="22">
+      <c r="F1" s="19" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="1" ht="54" hidden="1" spans="1:6">
+      <c r="A2" s="23">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="23" t="s">
+      <c r="B2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="24" t="s">
-        <v>7</v>
+      <c r="C2" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" ht="202.5" spans="1:5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" customFormat="1" ht="51" customHeight="1" spans="1:6">
       <c r="A3" s="25">
         <v>2</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" ht="40.5" spans="1:5">
-      <c r="A4" s="22">
+        <v>12</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="1" ht="54" hidden="1" spans="1:6">
+      <c r="A4" s="23">
         <v>3</v>
       </c>
-      <c r="B4" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" ht="162" spans="1:5">
+      <c r="B4" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" customFormat="1" ht="28" customHeight="1" spans="1:6">
       <c r="A5" s="25">
         <v>4</v>
       </c>
       <c r="B5" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="27" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" ht="67.5" spans="1:5">
-      <c r="A6" s="22">
+    </row>
+    <row r="6" customFormat="1" ht="108" hidden="1" spans="1:6">
+      <c r="A6" s="23">
         <v>5</v>
       </c>
-      <c r="B6" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" ht="40.5" spans="1:5">
+      <c r="B6" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="1" ht="33" customHeight="1" spans="1:6">
       <c r="A7" s="25">
         <v>6</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" ht="121.5" spans="1:5">
-      <c r="A8" s="22">
-        <v>7</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="30" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>23</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="1" ht="33" customHeight="1" spans="1:6">
+      <c r="A8" s="23">
+        <v>7</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" spans="1:6">
       <c r="A9" s="25">
         <v>8</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="31"/>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="22">
+        <v>11</v>
+      </c>
+      <c r="D9" s="30"/>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" customFormat="1" spans="1:6">
+      <c r="A10" s="23">
         <v>9</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="32"/>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="B10" s="24" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="30"/>
+      <c r="E10" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" customFormat="1" ht="18" customHeight="1" spans="1:6">
       <c r="A11" s="25">
         <v>10</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="31"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="22">
-        <v>11</v>
-      </c>
-      <c r="B12" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+      <c r="D11" s="30"/>
+      <c r="E11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F11" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" customFormat="1" ht="24" customHeight="1" spans="1:6">
+      <c r="A12" s="23">
+        <v>11</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>11</v>
       </c>
       <c r="D12" s="32"/>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="E12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" customFormat="1" ht="25" customHeight="1" spans="1:6">
       <c r="A13" s="25">
         <v>12</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C13" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="31"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="22">
+        <v>11</v>
+      </c>
+      <c r="D13" s="30"/>
+      <c r="E13" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" customFormat="1" ht="21" customHeight="1" spans="1:6">
+      <c r="A14" s="23">
         <v>13</v>
       </c>
-      <c r="B14" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="33" t="s">
-        <v>10</v>
+      <c r="B14" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>11</v>
       </c>
       <c r="D14" s="32"/>
-    </row>
-    <row r="15" ht="67.5" spans="1:5">
+      <c r="E14" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" ht="121.5" hidden="1" spans="1:6">
       <c r="A15" s="25">
         <v>14</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="22">
+        <v>39</v>
+      </c>
+      <c r="E15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" customFormat="1" ht="18" customHeight="1" spans="1:6">
+      <c r="A16" s="23">
         <v>15</v>
       </c>
-      <c r="B16" s="23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="30" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="B16" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="1" ht="29" customHeight="1" spans="1:6">
       <c r="A17" s="25">
         <v>16</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="31" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="22">
+        <v>11</v>
+      </c>
+      <c r="D17" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" customFormat="1" ht="23" customHeight="1" spans="1:6">
+      <c r="A18" s="23">
         <v>17</v>
       </c>
-      <c r="B18" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>10</v>
+      <c r="B18" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="D18" s="32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" ht="135" spans="1:4">
+        <v>42</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" customFormat="1" ht="23" customHeight="1" spans="1:6">
       <c r="A19" s="25">
         <v>18</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="22">
+        <v>11</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="E19" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" customFormat="1" hidden="1" spans="1:6">
+      <c r="A20" s="23">
         <v>19</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>6</v>
+      <c r="B20" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D20" s="32" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" customFormat="1" ht="23" customHeight="1" spans="1:6">
       <c r="A21" s="25">
         <v>20</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" s="31" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="22">
+        <v>11</v>
+      </c>
+      <c r="D21" s="30" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" customFormat="1" ht="20" customHeight="1" spans="1:6">
+      <c r="A22" s="23">
         <v>21</v>
       </c>
-      <c r="B22" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>10</v>
+      <c r="B22" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="D22" s="32" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>56</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F22" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" customFormat="1" ht="27" hidden="1" spans="1:6">
       <c r="A23" s="25">
         <v>22</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="31" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="22">
+        <v>7</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" customFormat="1" hidden="1" spans="1:6">
+      <c r="A24" s="23">
         <v>23</v>
       </c>
-      <c r="B24" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>6</v>
+      <c r="B24" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D24" s="32" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" customFormat="1" hidden="1" spans="1:6">
       <c r="A25" s="25">
         <v>24</v>
       </c>
       <c r="B25" s="26" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" s="31" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="22">
+        <v>7</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" customFormat="1" hidden="1" spans="1:6">
+      <c r="A26" s="23">
         <v>25</v>
       </c>
-      <c r="B26" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>6</v>
+      <c r="B26" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C26" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D26" s="32" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" customFormat="1" hidden="1" spans="1:6">
       <c r="A27" s="25">
         <v>26</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="31" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="22">
+        <v>7</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" customFormat="1" ht="27" hidden="1" spans="1:6">
+      <c r="A28" s="23">
         <v>27</v>
       </c>
-      <c r="B28" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="C28" s="23" t="s">
-        <v>6</v>
+      <c r="B28" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D28" s="32" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" customFormat="1" hidden="1" spans="1:6">
       <c r="A29" s="25">
         <v>28</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="31" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="22">
+        <v>7</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" customFormat="1" hidden="1" spans="1:6">
+      <c r="A30" s="23">
         <v>29</v>
       </c>
-      <c r="B30" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="C30" s="23" t="s">
-        <v>6</v>
+      <c r="B30" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D30" s="32" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="31" customFormat="1" hidden="1" spans="1:6">
       <c r="A31" s="25">
         <v>30</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="31" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="22">
+        <v>7</v>
+      </c>
+      <c r="D31" s="30" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="32" customFormat="1" hidden="1" spans="1:6">
+      <c r="A32" s="23">
         <v>31</v>
       </c>
-      <c r="B32" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="C32" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="B32" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D32" s="32" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33" customFormat="1" hidden="1" spans="1:6">
       <c r="A33" s="25">
         <v>32</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="22">
+        <v>7</v>
+      </c>
+      <c r="D33" s="30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="34" customFormat="1" hidden="1" spans="1:6">
+      <c r="A34" s="23">
         <v>33</v>
       </c>
-      <c r="B34" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="B34" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D34" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35" customFormat="1" hidden="1" spans="1:6">
       <c r="A35" s="25">
         <v>34</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>60</v>
+        <v>76</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="22">
+        <v>7</v>
+      </c>
+      <c r="D35" s="30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" customFormat="1" hidden="1" spans="1:6">
+      <c r="A36" s="23">
         <v>35</v>
       </c>
-      <c r="B36" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="B36" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="32" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="37" customFormat="1" hidden="1" spans="1:6">
       <c r="A37" s="25">
         <v>36</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" s="31" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="22">
+        <v>7</v>
+      </c>
+      <c r="D37" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" customFormat="1" hidden="1" spans="1:6">
+      <c r="A38" s="23">
         <v>37</v>
       </c>
-      <c r="B38" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C38" s="23" t="s">
-        <v>6</v>
+      <c r="B38" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D38" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" customFormat="1" hidden="1" spans="1:6">
       <c r="A39" s="25">
         <v>38</v>
       </c>
       <c r="B39" s="26" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" s="31" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="22">
+        <v>7</v>
+      </c>
+      <c r="D39" s="30" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="40" customFormat="1" hidden="1" spans="1:6">
+      <c r="A40" s="23">
         <v>39</v>
       </c>
-      <c r="B40" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="C40" s="23" t="s">
-        <v>6</v>
+      <c r="B40" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="C40" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D40" s="32" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="41" customFormat="1" ht="13" customHeight="1" spans="1:6">
       <c r="A41" s="25">
         <v>40</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="31" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="22">
+        <v>11</v>
+      </c>
+      <c r="D41" s="30" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41" t="s">
+        <v>85</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" customFormat="1" spans="1:6">
+      <c r="A42" s="23">
         <v>41</v>
       </c>
-      <c r="B42" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>10</v>
+      <c r="B42" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>11</v>
       </c>
       <c r="D42" s="32" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
+        <v>87</v>
+      </c>
+      <c r="E42" t="s">
+        <v>85</v>
+      </c>
+      <c r="F42" s="19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" customFormat="1" hidden="1" spans="1:6">
       <c r="A43" s="25">
         <v>42</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="31" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="22">
+        <v>7</v>
+      </c>
+      <c r="D43" s="30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" customFormat="1" hidden="1" spans="1:6">
+      <c r="A44" s="23">
         <v>43</v>
       </c>
-      <c r="B44" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="C44" s="23" t="s">
-        <v>6</v>
+      <c r="B44" s="24" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="24" t="s">
+        <v>7</v>
       </c>
       <c r="D44" s="32" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="34">
         <v>44</v>
       </c>
-      <c r="B45" s="36" t="s">
-        <v>74</v>
-      </c>
-      <c r="C45" s="36" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="37" t="s">
-        <v>75</v>
+      <c r="B45" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="36" t="s">
+        <v>92</v>
+      </c>
+      <c r="E45" t="s">
+        <v>93</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D45" etc:filterBottomFollowUsedRange="0">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="模型"/>
+      </filters>
+    </filterColumn>
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2415,16 +2616,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5" outlineLevelCol="4"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr defaultColWidth="9.025" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="5.51327433628319" customWidth="1"/>
-    <col min="2" max="2" width="25.3451327433628" customWidth="1"/>
-    <col min="3" max="3" width="11.5398230088496" customWidth="1"/>
-    <col min="4" max="4" width="59.283185840708" customWidth="1"/>
+    <col min="1" max="1" width="5.51666666666667" customWidth="1"/>
+    <col min="2" max="2" width="25.3416666666667" customWidth="1"/>
+    <col min="3" max="3" width="11.5416666666667" customWidth="1"/>
+    <col min="4" max="4" width="57.8333333333333" customWidth="1"/>
+    <col min="5" max="5" width="39.7333333333333" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2440,215 +2642,236 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" ht="40.5" spans="1:5">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="40.5" spans="1:6">
       <c r="A2" s="4">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>99</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" ht="27" spans="1:6">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+        <v>102</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" ht="67.5" spans="1:6">
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="B6" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
       <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="B7" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
       <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>6</v>
+      <c r="B8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>7</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
       <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="B9" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
       <c r="A10" s="4">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>86</v>
+        <v>107</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
       <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="B11" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
       <c r="A12" s="4">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
       <c r="A13" s="7">
         <v>12</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="B13" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
       <c r="A14" s="4">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>91</v>
+        <v>112</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
       <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="B15" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
       <c r="A16" s="4">
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>95</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-08-17 17:37:39
</commit_message>
<xml_diff>
--- a/工作交付文档/需求开发记录/assets/随州中心医院-住院病案附页-字段生成/V3366病案首页生成字段.xlsx
+++ b/工作交付文档/需求开发记录/assets/随州中心医院-住院病案附页-字段生成/V3366病案首页生成字段.xlsx
@@ -5,19 +5,20 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\gitee\obsidian_qyc_book\工作交付文档\需求开发记录\assets\随州中心医院-住院病案附页-字段生成\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rongz\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27705" windowHeight="12975" activeTab="1"/>
+    <workbookView windowWidth="21600" windowHeight="9555"/>
   </bookViews>
   <sheets>
     <sheet name="随州中心医院病案首页新加字段" sheetId="2" r:id="rId1"/>
     <sheet name="盐城中医院病案首页新加字段" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">随州中心医院病案首页新加字段!$A$1:$D$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">盐城中医院病案首页新加字段!$A$1:$D$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">随州中心医院病案首页新加字段!$C$1:$C$45</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="392">
   <si>
     <t>序号</t>
   </si>
@@ -55,6 +78,9 @@
   </si>
   <si>
     <t>负责人</t>
+  </si>
+  <si>
+    <t>负责人2</t>
   </si>
   <si>
     <t>是否急性ST段抬高型心肌梗死</t>
@@ -69,6 +95,9 @@
   </si>
   <si>
     <t>根据卫健委的定义。定制文案</t>
+  </si>
+  <si>
+    <t>邵帅</t>
   </si>
   <si>
     <t>急性ST段抬高型心肌梗死-再灌注治疗</t>
@@ -93,7 +122,7 @@
 （3）未执行：未在发病 12 小时内实施 PCI 或静脉溶栓。</t>
   </si>
   <si>
-    <t>入院记录，手术记录，操作记录，查房记录、日常病程记录
+    <t>入院记录，手术记录，操作记录（包含在日常病程记录表里了），查房记录、日常病程记录
 召召了解一下？填写的入口条件</t>
   </si>
   <si>
@@ -137,6 +166,9 @@
     <t>“肿瘤治疗前是否进行临床 TNM 分期“ 的区别</t>
   </si>
   <si>
+    <t>孙超</t>
+  </si>
+  <si>
     <t>肿瘤临床分期时间</t>
   </si>
   <si>
@@ -255,7 +287,7 @@
     <t>参考病历质控系统中制作的抗菌药物目录，是否病原学送检的提示词</t>
   </si>
   <si>
-    <t>病案质控中，我们做过了，有抗菌药物的收费项触发，查看医疗文本里是否有送检的相关描述</t>
+    <t>selectprompt_mark_dictWHEREtype=24; 存在抗菌药物就触发，手术记录+有创操作记录+检查报告（是操作记录的）</t>
   </si>
   <si>
     <t>有无输血反应</t>
@@ -266,6 +298,9 @@
   <si>
     <t>日常病程记录，查房记录
 召召了解一下？ 入口判断是否输过血（收费项目判断：红细胞、血小板、血浆、全血、自体回收、其他）</t>
+  </si>
+  <si>
+    <t>尹总</t>
   </si>
   <si>
     <t>红细胞</t>
@@ -445,6 +480,819 @@
   </si>
   <si>
     <t>与湖北版中抢救成功次数生成逻辑一样</t>
+  </si>
+  <si>
+    <t>结肠多发息肉（已钳除）</t>
+  </si>
+  <si>
+    <t>胃体息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃角溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>食管炎A级（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎（活检定性）</t>
+  </si>
+  <si>
+    <t>食管粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃角黄色素瘤（活检定性）</t>
+  </si>
+  <si>
+    <t>萎缩性胃炎伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠球部炎症、胃窦溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃角粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管炎A级、贲门粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>电子支气管镜检查+支气管镜诊断性肺泡灌洗术+吸痰术+镜下滴药</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下滴药</t>
+  </si>
+  <si>
+    <t>结肠多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠Ca（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术</t>
+  </si>
+  <si>
+    <t>萎缩性胃炎伴糜烂、胃角粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦多发溃疡(ForrestIII级)（活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>肛门隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎3级（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠炎（活检定性）</t>
+  </si>
+  <si>
+    <t>幽门粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜粘膜活检术+止血术+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+吸痰术</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜粘膜活检术+止血术+经纤支镜肺泡灌洗诊疗术+吸痰术</t>
+  </si>
+  <si>
+    <t>残胃粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>慢性非萎缩性胃炎伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃底息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>回盲瓣粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>横结肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃角-胃窦Ca（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>ERCP+EST+EPBD+球囊取石+ENBD</t>
+  </si>
+  <si>
+    <t>大肠多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端及回盲瓣粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>慢性萎缩性胃炎伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦多发溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体多发息肉切除术</t>
+  </si>
+  <si>
+    <t>食管乳头状瘤切除术</t>
+  </si>
+  <si>
+    <t>ERCP+EST+EPBD+网篮取石+球囊探查+ENBD</t>
+  </si>
+  <si>
+    <t>直肠息肉EMR术</t>
+  </si>
+  <si>
+    <t>结肠多发息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>回盲部息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎2级（肠化？活检定性）</t>
+  </si>
+  <si>
+    <t>胃体病变病变（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端粘膜改变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦黄色素瘤（活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>升结肠Ca（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+吸痰术</t>
+  </si>
+  <si>
+    <t>降结肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>慢性萎缩性胃炎（C3）伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉内镜下切除术（CSP）</t>
+  </si>
+  <si>
+    <t>直肠粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦溃疡（Ca？活检定性）</t>
+  </si>
+  <si>
+    <t>结肠息肉APC术</t>
+  </si>
+  <si>
+    <t>（横结肠+降结肠）息肉EMR术</t>
+  </si>
+  <si>
+    <t>乙状结肠隆起（炎症？活检定性）</t>
+  </si>
+  <si>
+    <t>贲门微隆起（息肉？钳除</t>
+  </si>
+  <si>
+    <t>食管隆起（乳头状瘤？活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉、直肠隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>直乙交界处隆起（绒面管状腺瘤？活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>十二指肠球部炎症、糜烂性胃炎（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠隆起EMR术</t>
+  </si>
+  <si>
+    <t>食管炎（活检定性）</t>
+  </si>
+  <si>
+    <t>食管异物内镜下取出术</t>
+  </si>
+  <si>
+    <t>胃体黄色素瘤（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体息肉切除术（CSP+APC）</t>
+  </si>
+  <si>
+    <t>胃粘膜病变EMR术</t>
+  </si>
+  <si>
+    <t>直肠粘膜溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>直肠术后;吻合口出血止血术</t>
+  </si>
+  <si>
+    <t>结肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉切除术</t>
+  </si>
+  <si>
+    <t>回盲瓣、直肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管中段白色隆起（乳头状瘤、钳除</t>
+  </si>
+  <si>
+    <t>胃多发息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>食管静脉曲张破裂出血硬化治疗</t>
+  </si>
+  <si>
+    <t>胃角、胃体粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉冷圈套切除术（CSP）</t>
+  </si>
+  <si>
+    <t>升结肠隆起EMR术</t>
+  </si>
+  <si>
+    <t>结肠多发息肉高频电凝切除术</t>
+  </si>
+  <si>
+    <t>胃窦息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>降结肠息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉EMR术</t>
+  </si>
+  <si>
+    <t>降结肠息肉切除（CSP）</t>
+  </si>
+  <si>
+    <t>乙状结肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>溃疡性直肠炎（活检定性）</t>
+  </si>
+  <si>
+    <t>窦体交界隆起（息肉？活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠球部息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下止血+镜下滴药；</t>
+  </si>
+  <si>
+    <t>十二指肠球部出血内镜下止血治疗</t>
+  </si>
+  <si>
+    <t>横结肠息肉EMR术</t>
+  </si>
+  <si>
+    <t>升结肠息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>乙状结肠新生物（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉EMR术</t>
+  </si>
+  <si>
+    <t>结肠多发长蒂息肉HSP</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉切除术（HSP）</t>
+  </si>
+  <si>
+    <t>升结肠息肉内镜下切除术（CSP）</t>
+  </si>
+  <si>
+    <t>胃体息肉、食管胃粘膜异位（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下滴药</t>
+  </si>
+  <si>
+    <t>主支气管下端右侧粘膜刷检</t>
+  </si>
+  <si>
+    <t>胃多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>食管息肉EMR术</t>
+  </si>
+  <si>
+    <t>食管下段粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门多发息肉切除术</t>
+  </si>
+  <si>
+    <t>胃底息肉切除术</t>
+  </si>
+  <si>
+    <t>Barrett食管、食管粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门炎（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎2级、胃体粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管炎A级、十二指肠降部隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>横结肠息肉冷圈套切除术（CSP）</t>
+  </si>
+  <si>
+    <t>横结肠多发息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>胃底多发息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>十二指肠球部霜斑样溃疡、糜烂性胃炎2级（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠息肉（活检定性</t>
+  </si>
+  <si>
+    <t>十二指肠降部粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>回盲部多发息肉切除术</t>
+  </si>
+  <si>
+    <t>胃角溃疡（Ca？活检定性）</t>
+  </si>
+  <si>
+    <t>食管血管畸形止血术</t>
+  </si>
+  <si>
+    <t>胃底、胃体息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>幽门粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管胃粘膜异位（活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠异物取出术</t>
+  </si>
+  <si>
+    <t>结直肠息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>右半结肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>鼻胃管置入胃窦术</t>
+  </si>
+  <si>
+    <t>胃底息肉、食管炎(活检定性)</t>
+  </si>
+  <si>
+    <t>食管隆起出血止血术</t>
+  </si>
+  <si>
+    <t>回肠末端溃疡（CD?活检定性）</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉冷圈套切除术（CSP）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜粘膜活检术+止血术+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下滴药</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉、乙状结肠隆起（肉芽肿？活检定性）</t>
+  </si>
+  <si>
+    <t>ERCP+EPBD+球囊取石+ENBD</t>
+  </si>
+  <si>
+    <t>胃体息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>十二指肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>萎缩性胃炎（活检定性）</t>
+  </si>
+  <si>
+    <t>升结肠黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>食管隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉切除术（EMR+CSP）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉EMR+CSP</t>
+  </si>
+  <si>
+    <t>纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术</t>
+  </si>
+  <si>
+    <t>乙状结肠Ca（活检定性）</t>
+  </si>
+  <si>
+    <t>ERCP+ERPD</t>
+  </si>
+  <si>
+    <t>胃体隆起EMR术</t>
+  </si>
+  <si>
+    <t>乙状结肠、直肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎2级、幽门粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体息肉、胃体黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>升结肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直乙交界处多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠LSTESD术</t>
+  </si>
+  <si>
+    <t>十二指肠降部多发隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>升结肠溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠息肉冷圈套切除术(CSP)</t>
+  </si>
+  <si>
+    <t>食管静脉曲张套扎术</t>
+  </si>
+  <si>
+    <t>回结肠多发息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>结肠多发息肉、回盲部隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体APC术</t>
+  </si>
+  <si>
+    <t>结肠多发息肉EMR+电凝切除</t>
+  </si>
+  <si>
+    <t>升结肠息肉冷圈套切除术（CSP）</t>
+  </si>
+  <si>
+    <t>升结肠隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉、直肠粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃底静脉曲张破裂出血止血术（硬化注射术）</t>
+  </si>
+  <si>
+    <t>横结肠息肉切除术(CSP)</t>
+  </si>
+  <si>
+    <t>食管内异物取出术</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉切除术（APC术）</t>
+  </si>
+  <si>
+    <t>大肠多发息肉EMR/高频电凝摘除</t>
+  </si>
+  <si>
+    <t>升结肠息肉（钳除</t>
+  </si>
+  <si>
+    <t>横降交界处粘膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉切除术(CSP+CFP)</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术+经纤支镜滴药</t>
+  </si>
+  <si>
+    <t>胃体溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎、食管炎B级、贲门炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠多发息肉、横结肠黏膜炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>US—FNA：（左锁骨上淋巴结）</t>
+  </si>
+  <si>
+    <t>ERCP+EST+EPBD+球囊取石+ERPD+ENBD</t>
+  </si>
+  <si>
+    <t>回盲部粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>回盲瓣粘膜改变（活检定性）</t>
+  </si>
+  <si>
+    <t>大肠息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+止血术+吸痰术+镜下滴药</t>
+  </si>
+  <si>
+    <t>横结肠多发息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体多发息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>横结肠息肉、直肠隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦黄色素瘤切除术</t>
+  </si>
+  <si>
+    <t>浅表糜烂性胃炎、胃窦浅溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃窦Ca（活检定性）</t>
+  </si>
+  <si>
+    <t>胃多发息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>直肠粘膜改变（活检定性）</t>
+  </si>
+  <si>
+    <t>ERCP+EPBD+网篮取石+球囊探查+ENBD</t>
+  </si>
+  <si>
+    <t>结肠多发息肉高频电凝切除术（HSP）</t>
+  </si>
+  <si>
+    <t>ERCP+EST</t>
+  </si>
+  <si>
+    <t>直肠APC术</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎2级、胃窦粘膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>胃体息肉内镜下切除术</t>
+  </si>
+  <si>
+    <t>贲门溃疡（ForrestIII级）（活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠息肉切除术</t>
+  </si>
+  <si>
+    <t>十二指肠降部炎症改变（活检定性）</t>
+  </si>
+  <si>
+    <t>肛周隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉氩离子凝固术APC+CSP</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎并小球样隆起（息肉、钳除</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜活检术+经纤支镜防污染采样刷检查+经纤支镜肺泡灌洗诊疗术+止血术+吸痰术</t>
+  </si>
+  <si>
+    <t>降结肠息肉CSP</t>
+  </si>
+  <si>
+    <t>胃底黏膜病变（活检定性）</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>胃角息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠球部息肉切除术（CSP）</t>
+  </si>
+  <si>
+    <t>升结肠憩室、肝区息肉（活检定性）</t>
+  </si>
+  <si>
+    <t>回肠末端多发溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>横结肠息肉切除术(CFP)</t>
+  </si>
+  <si>
+    <t>幽门溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>贲门溃疡出血止血术</t>
+  </si>
+  <si>
+    <t>胃底小球样隆起（息肉、钳除</t>
+  </si>
+  <si>
+    <t>食管隆起切除术</t>
+  </si>
+  <si>
+    <t>胃体息肉切除术</t>
+  </si>
+  <si>
+    <t>胃镜下十二指肠置管术</t>
+  </si>
+  <si>
+    <t>胃窦隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>十二指肠隆起（活检定性）</t>
+  </si>
+  <si>
+    <t>结肠息肉高频电凝切除术</t>
+  </si>
+  <si>
+    <t>乙状结肠APC术</t>
+  </si>
+  <si>
+    <t>乙状结肠息肉，回盲瓣溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>胃多发息肉切除术</t>
+  </si>
+  <si>
+    <t>胃镜下空肠置管术</t>
+  </si>
+  <si>
+    <t>直肠肿物（Ca？活检定性）</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下滴药止血</t>
+  </si>
+  <si>
+    <t>慢性萎缩性胃炎（A型胃炎？）伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>结直肠多发息肉切除术（APC）</t>
+  </si>
+  <si>
+    <t>直肠息肉高频电凝切除术</t>
+  </si>
+  <si>
+    <t>降结肠息肉EMR术</t>
+  </si>
+  <si>
+    <t>萎缩性胃炎（C2）（活检定性）</t>
+  </si>
+  <si>
+    <t>升结肠息肉EMR术</t>
+  </si>
+  <si>
+    <t>升结肠息肉电凝切除术</t>
+  </si>
+  <si>
+    <t>电子纤维支气管镜检查+经纤支镜肺泡灌洗诊疗术+吸痰术+镜下止血+镜下滴药</t>
+  </si>
+  <si>
+    <t>食管炎（霉菌性？）（活检定性）</t>
+  </si>
+  <si>
+    <t>升结肠肿瘤（性质待定）</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎并溃疡（性质待查）</t>
+  </si>
+  <si>
+    <t>直肠多发息肉APC术</t>
+  </si>
+  <si>
+    <t>升结肠息肉EMR术+电凝切除术</t>
+  </si>
+  <si>
+    <t>A型胃炎？（活检定性）</t>
+  </si>
+  <si>
+    <t>直肠多发息肉内镜下切除术</t>
+  </si>
+  <si>
+    <t>糜烂性胃炎、胃窦溃疡（活检定性）</t>
+  </si>
+  <si>
+    <t>慢性萎缩性胃炎（C1）伴糜烂（活检定性）</t>
+  </si>
+  <si>
+    <t>胃底-胃体多发息肉高频电凝切除术</t>
+  </si>
+  <si>
+    <t>升结肠多发息肉EMR术</t>
+  </si>
+  <si>
+    <t>升结肠息肉高频电凝切除术</t>
   </si>
 </sst>
 </file>
@@ -1204,7 +2052,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1295,17 +2143,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1840,19 +2682,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:F45"/>
-  <sheetFormatPr defaultColWidth="9.025" defaultRowHeight="13.5" outlineLevelCol="5"/>
+  <sheetPr/>
+  <dimension ref="A1:G45"/>
+  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="7.41666666666667" style="18" customWidth="1"/>
-    <col min="2" max="2" width="33.7916666666667" style="18" customWidth="1"/>
-    <col min="3" max="3" width="9.225" style="18" customWidth="1"/>
-    <col min="4" max="4" width="45.0916666666667" style="12" customWidth="1"/>
-    <col min="5" max="5" width="41.6333333333333" customWidth="1"/>
-    <col min="6" max="6" width="9.025" style="19"/>
+    <col min="1" max="1" width="7.41592920353982" style="18" customWidth="1"/>
+    <col min="2" max="2" width="33.787610619469" style="18" customWidth="1"/>
+    <col min="3" max="3" width="9.2212389380531" style="18" customWidth="1"/>
+    <col min="4" max="4" width="29.6637168141593" style="12" customWidth="1"/>
+    <col min="5" max="5" width="39.5663716814159" customWidth="1"/>
+    <col min="6" max="6" width="10.7345132743363" style="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" spans="1:6">
+    <row r="1" customFormat="1" spans="1:7">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -1871,743 +2713,870 @@
       <c r="F1" s="19" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" customFormat="1" ht="54" hidden="1" spans="1:6">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" customFormat="1" ht="81" spans="1:7">
       <c r="A2" s="23">
         <v>1</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" customFormat="1" ht="51" customHeight="1" spans="1:6">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="1" ht="51" customHeight="1" spans="1:7">
       <c r="A3" s="25">
         <v>2</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" customFormat="1" ht="54" hidden="1" spans="1:6">
+    </row>
+    <row r="4" customFormat="1" ht="81" spans="1:7">
       <c r="A4" s="23">
         <v>3</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" customFormat="1" ht="28" customHeight="1" spans="1:6">
+        <v>18</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="1" ht="28" customHeight="1" spans="1:7">
       <c r="A5" s="25">
         <v>4</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C5" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" customFormat="1" ht="108" hidden="1" spans="1:6">
+    </row>
+    <row r="6" customFormat="1" ht="148.5" spans="1:7">
       <c r="A6" s="23">
         <v>5</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" customFormat="1" ht="33" customHeight="1" spans="1:6">
+        <v>23</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="1" ht="49" customHeight="1" spans="1:7">
       <c r="A7" s="25">
         <v>6</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C7" s="28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" customFormat="1" ht="33" customHeight="1" spans="1:6">
+    </row>
+    <row r="8" customFormat="1" ht="33" customHeight="1" spans="1:7">
       <c r="A8" s="23">
         <v>7</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" customFormat="1" spans="1:6">
+        <v>31</v>
+      </c>
+      <c r="G8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" customFormat="1" spans="1:7">
       <c r="A9" s="25">
         <v>8</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="30"/>
+        <v>13</v>
+      </c>
+      <c r="D9" s="27"/>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" customFormat="1" spans="1:6">
+        <v>31</v>
+      </c>
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" customFormat="1" spans="1:7">
       <c r="A10" s="23">
         <v>9</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="27"/>
+      <c r="E10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="30"/>
-      <c r="E10" t="s">
-        <v>27</v>
-      </c>
       <c r="F10" s="19" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" customFormat="1" ht="18" customHeight="1" spans="1:6">
+        <v>31</v>
+      </c>
+      <c r="G10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" customFormat="1" ht="18" customHeight="1" spans="1:7">
       <c r="A11" s="25">
         <v>10</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C11" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="30"/>
+        <v>13</v>
+      </c>
+      <c r="D11" s="27"/>
       <c r="E11" s="12" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" customFormat="1" ht="24" customHeight="1" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="G11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" customFormat="1" ht="24" customHeight="1" spans="1:7">
       <c r="A12" s="23">
         <v>11</v>
       </c>
-      <c r="B12" s="31" t="s">
-        <v>34</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="32"/>
+      <c r="B12" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="6"/>
       <c r="E12" s="12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" customFormat="1" ht="25" customHeight="1" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="G12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" customFormat="1" ht="25" customHeight="1" spans="1:7">
       <c r="A13" s="25">
         <v>12</v>
       </c>
       <c r="B13" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="27"/>
+      <c r="E13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C13" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="30"/>
-      <c r="E13" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" customFormat="1" ht="21" customHeight="1" spans="1:6">
+      <c r="G13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" customFormat="1" ht="21" customHeight="1" spans="1:7">
       <c r="A14" s="23">
         <v>13</v>
       </c>
-      <c r="B14" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="31" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="32"/>
+      <c r="B14" s="30" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="6"/>
       <c r="E14" s="12" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" customFormat="1" ht="121.5" hidden="1" spans="1:6">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" customFormat="1" ht="148.5" spans="1:7">
       <c r="A15" s="25">
         <v>14</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" s="27" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" customFormat="1" ht="18" customHeight="1" spans="1:6">
+        <v>43</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="1" ht="18" customHeight="1" spans="1:7">
       <c r="A16" s="23">
         <v>15</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C16" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" t="s">
         <v>11</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E16" t="s">
-        <v>43</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" customFormat="1" ht="29" customHeight="1" spans="1:6">
+    </row>
+    <row r="17" customFormat="1" ht="29" customHeight="1" spans="1:7">
       <c r="A17" s="25">
         <v>16</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C17" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F17" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="30" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" customFormat="1" ht="23" customHeight="1" spans="1:6">
+    </row>
+    <row r="18" customFormat="1" ht="23" customHeight="1" spans="1:7">
       <c r="A18" s="23">
         <v>17</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C18" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" t="s">
         <v>11</v>
       </c>
-      <c r="D18" s="32" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="F18" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" customFormat="1" ht="23" customHeight="1" spans="1:6">
+    </row>
+    <row r="19" customFormat="1" ht="23" customHeight="1" spans="1:7">
       <c r="A19" s="25">
         <v>18</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C19" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" t="s">
+        <v>52</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="27" t="s">
-        <v>48</v>
-      </c>
-      <c r="E19" t="s">
-        <v>49</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" customFormat="1" hidden="1" spans="1:6">
+    </row>
+    <row r="20" customFormat="1" ht="27" spans="1:7">
       <c r="A20" s="23">
         <v>19</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="32" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="21" customFormat="1" ht="23" customHeight="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="1" ht="52" customHeight="1" spans="1:7">
       <c r="A21" s="25">
         <v>20</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C21" s="26" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" t="s">
         <v>11</v>
       </c>
-      <c r="D21" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="E21" s="33" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" customFormat="1" ht="20" customHeight="1" spans="1:6">
+    </row>
+    <row r="22" customFormat="1" ht="20" customHeight="1" spans="1:7">
       <c r="A22" s="23">
         <v>21</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="32" t="s">
-        <v>56</v>
+        <v>13</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>59</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" customFormat="1" ht="27" hidden="1" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="G22" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="23" customFormat="1" ht="27" spans="1:7">
       <c r="A23" s="25">
         <v>22</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D23" s="30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="24" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="G23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" customFormat="1" ht="27" spans="1:7">
       <c r="A24" s="23">
         <v>23</v>
       </c>
       <c r="B24" s="24" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C24" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="32" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="25" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="25" customFormat="1" ht="27" spans="1:7">
       <c r="A25" s="25">
         <v>24</v>
       </c>
       <c r="B25" s="26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C25" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="27" t="s">
+        <v>63</v>
+      </c>
+      <c r="G25" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="30" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" customFormat="1" hidden="1" spans="1:6">
+    </row>
+    <row r="26" customFormat="1" ht="27" spans="1:7">
       <c r="A26" s="23">
         <v>25</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C26" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="32" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G26" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="27" customFormat="1" spans="1:7">
       <c r="A27" s="25">
         <v>26</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="30" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="28" customFormat="1" ht="27" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>68</v>
+      </c>
+      <c r="G27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" customFormat="1" ht="27" spans="1:7">
       <c r="A28" s="23">
         <v>27</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C28" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D28" s="32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="29" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G28" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" customFormat="1" spans="1:7">
       <c r="A29" s="25">
         <v>28</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D29" s="30" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="30" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G29" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="30" customFormat="1" spans="1:7">
       <c r="A30" s="23">
         <v>29</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="32" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="31" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" customFormat="1" spans="1:7">
       <c r="A31" s="25">
         <v>30</v>
       </c>
       <c r="B31" s="26" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="30" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="32" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>72</v>
+      </c>
+      <c r="G31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" customFormat="1" ht="27" spans="1:7">
       <c r="A32" s="23">
         <v>31</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C32" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D32" s="32" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="33" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="G32" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33" customFormat="1" ht="27" spans="1:7">
       <c r="A33" s="25">
         <v>32</v>
       </c>
       <c r="B33" s="26" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="30" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="34" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D33" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="G33" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="34" customFormat="1" ht="27" spans="1:7">
       <c r="A34" s="23">
         <v>33</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D34" s="32" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="35" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G34" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="35" customFormat="1" ht="27" spans="1:7">
       <c r="A35" s="25">
         <v>34</v>
       </c>
       <c r="B35" s="26" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D35" s="30" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="36" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D35" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="G35" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="36" customFormat="1" ht="27" spans="1:7">
       <c r="A36" s="23">
         <v>35</v>
       </c>
       <c r="B36" s="24" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C36" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="32" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="37" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G36" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" customFormat="1" spans="1:7">
       <c r="A37" s="25">
         <v>36</v>
       </c>
       <c r="B37" s="26" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D37" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="38" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="G37" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="38" customFormat="1" spans="1:7">
       <c r="A38" s="23">
         <v>37</v>
       </c>
       <c r="B38" s="24" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C38" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D38" s="32" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="39" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G38" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="39" customFormat="1" spans="1:7">
       <c r="A39" s="25">
         <v>38</v>
       </c>
       <c r="B39" s="26" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C39" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39" s="30" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="40" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="G39" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="40" customFormat="1" spans="1:7">
       <c r="A40" s="23">
         <v>39</v>
       </c>
       <c r="B40" s="24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C40" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D40" s="32" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" customFormat="1" ht="13" customHeight="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="G40" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" customFormat="1" ht="13" customHeight="1" spans="1:7">
       <c r="A41" s="25">
         <v>40</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C41" s="26" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="30" t="s">
-        <v>84</v>
+        <v>13</v>
+      </c>
+      <c r="D41" s="27" t="s">
+        <v>88</v>
       </c>
       <c r="E41" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" customFormat="1" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="G41" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="42" customFormat="1" spans="1:7">
       <c r="A42" s="23">
         <v>41</v>
       </c>
       <c r="B42" s="24" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C42" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" s="32" t="s">
-        <v>87</v>
+        <v>13</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="E42" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" customFormat="1" hidden="1" spans="1:6">
+        <v>16</v>
+      </c>
+      <c r="G42" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="43" customFormat="1" spans="1:7">
       <c r="A43" s="25">
         <v>42</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C43" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="30" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" customFormat="1" hidden="1" spans="1:6">
+        <v>8</v>
+      </c>
+      <c r="D43" s="27" t="s">
+        <v>93</v>
+      </c>
+      <c r="G43" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="44" customFormat="1" spans="1:7">
       <c r="A44" s="23">
         <v>43</v>
       </c>
       <c r="B44" s="24" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C44" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" s="32" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="34">
+        <v>8</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G44" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="45" ht="27" spans="1:7">
+      <c r="A45" s="32">
         <v>44</v>
       </c>
-      <c r="B45" s="35" t="s">
-        <v>91</v>
-      </c>
-      <c r="C45" s="35" t="s">
-        <v>11</v>
-      </c>
-      <c r="D45" s="36" t="s">
-        <v>92</v>
+      <c r="B45" s="33" t="s">
+        <v>95</v>
+      </c>
+      <c r="C45" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D45" s="34" t="s">
+        <v>96</v>
       </c>
       <c r="E45" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="G45" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:D45" etc:filterBottomFollowUsedRange="0">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="模型"/>
-      </filters>
-    </filterColumn>
-    <extLst/>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -2617,13 +3586,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultColWidth="9.025" defaultRowHeight="13.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="5.51666666666667" customWidth="1"/>
-    <col min="2" max="2" width="25.3416666666667" customWidth="1"/>
-    <col min="3" max="3" width="11.5416666666667" customWidth="1"/>
-    <col min="4" max="4" width="57.8333333333333" customWidth="1"/>
-    <col min="5" max="5" width="39.7333333333333" customWidth="1"/>
+    <col min="1" max="1" width="5.51327433628319" customWidth="1"/>
+    <col min="2" max="2" width="25.3451327433628" customWidth="1"/>
+    <col min="3" max="3" width="11.5398230088496" customWidth="1"/>
+    <col min="4" max="4" width="57.8318584070796" customWidth="1"/>
+    <col min="5" max="5" width="39.7345132743363" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2651,13 +3620,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -2665,13 +3634,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2679,19 +3648,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" ht="27" spans="1:6">
@@ -2699,19 +3668,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" ht="67.5" spans="1:6">
@@ -2719,19 +3688,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2739,13 +3708,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2753,13 +3722,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2767,13 +3736,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2781,13 +3750,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2795,13 +3764,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2809,13 +3778,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2823,13 +3792,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2837,13 +3806,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="17" t="s">
         <v>112</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2851,13 +3820,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2865,13 +3834,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -2881,4 +3850,1380 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:A272"/>
+  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="1" width="53.6991150442478" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="e" cm="1">
+        <f t="array" ref="A100">+直肠息肉APC术</f>
+        <v>#NAME?</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1">
+      <c r="A103" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1">
+      <c r="A104" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1">
+      <c r="A105" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1">
+      <c r="A106" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1">
+      <c r="A107" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1">
+      <c r="A108" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1">
+      <c r="A109" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1">
+      <c r="A110" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1">
+      <c r="A111" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1">
+      <c r="A112" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1">
+      <c r="A113" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1">
+      <c r="A114" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1">
+      <c r="A115" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1">
+      <c r="A116" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1">
+      <c r="A117" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1">
+      <c r="A118" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1">
+      <c r="A119" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1">
+      <c r="A120" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1">
+      <c r="A121" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1">
+      <c r="A122" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1">
+      <c r="A123" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1">
+      <c r="A124" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1">
+      <c r="A125" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1">
+      <c r="A126" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1">
+      <c r="A127" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1">
+      <c r="A128" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1">
+      <c r="A129" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1">
+      <c r="A130" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1">
+      <c r="A131" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1">
+      <c r="A132" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1">
+      <c r="A133" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1">
+      <c r="A134" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1">
+      <c r="A135" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1">
+      <c r="A136" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1">
+      <c r="A137" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1">
+      <c r="A138" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1">
+      <c r="A139" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1">
+      <c r="A140" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1">
+      <c r="A141" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1">
+      <c r="A142" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1">
+      <c r="A143" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1">
+      <c r="A144" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="145" spans="1:1">
+      <c r="A145" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1">
+      <c r="A146" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1">
+      <c r="A147" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="148" spans="1:1">
+      <c r="A148" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="149" spans="1:1">
+      <c r="A149" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="150" spans="1:1">
+      <c r="A150" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="151" spans="1:1">
+      <c r="A151" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="152" spans="1:1">
+      <c r="A152" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="153" spans="1:1">
+      <c r="A153" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="154" spans="1:1">
+      <c r="A154" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="155" spans="1:1">
+      <c r="A155" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="156" spans="1:1">
+      <c r="A156" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="157" spans="1:1">
+      <c r="A157" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="158" spans="1:1">
+      <c r="A158" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="159" spans="1:1">
+      <c r="A159" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="160" spans="1:1">
+      <c r="A160" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="161" spans="1:1">
+      <c r="A161" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="162" spans="1:1">
+      <c r="A162" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="163" spans="1:1">
+      <c r="A163" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="164" spans="1:1">
+      <c r="A164" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="165" spans="1:1">
+      <c r="A165" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="166" spans="1:1">
+      <c r="A166" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="167" spans="1:1">
+      <c r="A167" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="168" spans="1:1">
+      <c r="A168" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="169" spans="1:1">
+      <c r="A169" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="170" spans="1:1">
+      <c r="A170" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="171" spans="1:1">
+      <c r="A171" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="172" spans="1:1">
+      <c r="A172" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="173" spans="1:1">
+      <c r="A173" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="174" spans="1:1">
+      <c r="A174" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="175" spans="1:1">
+      <c r="A175" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="176" spans="1:1">
+      <c r="A176" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="177" spans="1:1">
+      <c r="A177" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="178" spans="1:1">
+      <c r="A178" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="179" spans="1:1">
+      <c r="A179" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="180" spans="1:1">
+      <c r="A180" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="181" spans="1:1">
+      <c r="A181" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="182" spans="1:1">
+      <c r="A182" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="183" spans="1:1">
+      <c r="A183" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="184" spans="1:1">
+      <c r="A184" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="185" spans="1:1">
+      <c r="A185" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="186" spans="1:1">
+      <c r="A186" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="187" spans="1:1">
+      <c r="A187" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="188" spans="1:1">
+      <c r="A188" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="189" spans="1:1">
+      <c r="A189" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="190" spans="1:1">
+      <c r="A190" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="191" spans="1:1">
+      <c r="A191" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="192" spans="1:1">
+      <c r="A192" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="193" spans="1:1">
+      <c r="A193" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="194" spans="1:1">
+      <c r="A194" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="195" spans="1:1">
+      <c r="A195" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="196" spans="1:1">
+      <c r="A196" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="197" spans="1:1">
+      <c r="A197" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="198" spans="1:1">
+      <c r="A198" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="199" spans="1:1">
+      <c r="A199" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="200" spans="1:1">
+      <c r="A200" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="201" spans="1:1">
+      <c r="A201" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="202" spans="1:1">
+      <c r="A202" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="203" spans="1:1">
+      <c r="A203" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="204" spans="1:1">
+      <c r="A204" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="205" spans="1:1">
+      <c r="A205" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="206" spans="1:1">
+      <c r="A206" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="207" spans="1:1">
+      <c r="A207" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="208" spans="1:1">
+      <c r="A208" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="209" spans="1:1">
+      <c r="A209" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="210" spans="1:1">
+      <c r="A210" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="211" spans="1:1">
+      <c r="A211" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="212" spans="1:1">
+      <c r="A212" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="213" spans="1:1">
+      <c r="A213" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="214" spans="1:1">
+      <c r="A214" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="215" spans="1:1">
+      <c r="A215" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="216" spans="1:1">
+      <c r="A216" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="217" spans="1:1">
+      <c r="A217" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="218" spans="1:1">
+      <c r="A218" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="219" spans="1:1">
+      <c r="A219" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="220" spans="1:1">
+      <c r="A220" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="221" spans="1:1">
+      <c r="A221" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="222" spans="1:1">
+      <c r="A222" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="223" spans="1:1">
+      <c r="A223" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="224" spans="1:1">
+      <c r="A224" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1">
+      <c r="A225" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="226" spans="1:1">
+      <c r="A226" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="227" spans="1:1">
+      <c r="A227" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="228" spans="1:1">
+      <c r="A228" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="229" spans="1:1">
+      <c r="A229" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="230" spans="1:1">
+      <c r="A230" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="231" spans="1:1">
+      <c r="A231" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="232" spans="1:1">
+      <c r="A232" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="233" spans="1:1">
+      <c r="A233" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="234" spans="1:1">
+      <c r="A234" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="235" spans="1:1">
+      <c r="A235" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="236" spans="1:1">
+      <c r="A236" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="237" spans="1:1">
+      <c r="A237" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="238" spans="1:1">
+      <c r="A238" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="239" spans="1:1">
+      <c r="A239" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="240" spans="1:1">
+      <c r="A240" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="241" spans="1:1">
+      <c r="A241" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="242" spans="1:1">
+      <c r="A242" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="243" spans="1:1">
+      <c r="A243" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="244" spans="1:1">
+      <c r="A244" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="245" spans="1:1">
+      <c r="A245" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="246" spans="1:1">
+      <c r="A246" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="247" spans="1:1">
+      <c r="A247" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="248" spans="1:1">
+      <c r="A248" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="249" spans="1:1">
+      <c r="A249" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="250" spans="1:1">
+      <c r="A250" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="251" spans="1:1">
+      <c r="A251" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="252" spans="1:1">
+      <c r="A252" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="253" spans="1:1">
+      <c r="A253" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="254" spans="1:1">
+      <c r="A254" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="255" spans="1:1">
+      <c r="A255" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="256" spans="1:1">
+      <c r="A256" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="257" spans="1:1">
+      <c r="A257" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="258" spans="1:1">
+      <c r="A258" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="259" spans="1:1">
+      <c r="A259" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="260" spans="1:1">
+      <c r="A260" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="261" spans="1:1">
+      <c r="A261" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="262" spans="1:1">
+      <c r="A262" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="263" spans="1:1">
+      <c r="A263" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="264" spans="1:1">
+      <c r="A264" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="265" spans="1:1">
+      <c r="A265" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="266" spans="1:1">
+      <c r="A266" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="267" spans="1:1">
+      <c r="A267" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="268" spans="1:1">
+      <c r="A268" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="269" spans="1:1">
+      <c r="A269" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="270" spans="1:1">
+      <c r="A270" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="271" spans="1:1">
+      <c r="A271" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="272" spans="1:1">
+      <c r="A272" t="s">
+        <v>391</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>